<commit_message>
chore: bump dr repo and generate reports
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
+++ b/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>225547.98</v>
+        <v>147764.16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>225547.98</v>
+        <v>147764.16</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
chore(dr): bump settle-dr-dune to 2a4e204 + refresh Skybase DR (#141)
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
+++ b/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
@@ -507,13 +507,13 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>225547.98</v>
+        <v>147764.16</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr"/>
       <c r="B7" s="4" t="n">
-        <v>225547.98</v>
+        <v>147764.16</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
feat(skybase): migrate debt+balance from Dune to Envio HyperSync
Skybase onto the HyperSync backend (sources: debt+balance). Agent-rate-only,
so debt is a no-op; balance reconstructs the subproxy USDS/sUSDS agent-rate
base from raw Transfer logs via the reorg-safe store. Prices/SSR/DR unchanged.

Parity: all 6 months (2026-01..06) regenerate byte-identical summary.md vs
Dune; .xlsx differ only in the regeneration timestamp.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
+++ b/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -624,7 +624,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:46+00:00</t>
+          <t>2026-07-14T09:34:21+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(gar): same-month SNR basis — month-N report carries 1% x SNR(N), paid at the MSC in N+1
Operator correction 2026-08-06: the GAR reported for July 2026 is paid
in August as part of MSC#11, so the July report's GAR = 1% x JULY's SNR
(not the prior month's). Still non-circular: SNR(N) is paid-basis and
carries the settlement executed IN month N (cycle N-1's payments), so it
never contains month N's own GAR; the GAR(N) cash reduces SNR(N+1)
through the normal subproxy-send subtraction.

January now computes normally (1% x Jan SNR = 92,187.14) instead of
rendering N/A - under the same-month basis no 2025-12 artifact is
needed; the dead N/A branch and its render path are removed. Full
series: Jan 92,187.14 / Feb 331,414.43 / Mar 218,409.05 / Apr
124,885.03 / May 140,660.93 / Jun 148,750.75 / Jul 152,255.89.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
+++ b/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -511,130 +511,140 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>222064.54</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>+ governance_accessibility_rewards (0.01 × SNR 2026-01 = 9218713.81273186308887946403 (sky_total generated sky_total))</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>92187.13812731863</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" s="4" t="n">
+        <v>314251.6781273186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-01-01 → 2026-01-31 (31 days)</t>
-        </is>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ethereum=24358292</t>
+          <t>2026-01-01 → 2026-01-31 (31 days)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-05T23:50:42+00:00</t>
+          <t>ethereum=24358292</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-06T00:02:30+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>

<commit_message>
fix(gar): same-month SNR basis — July's GAR (1% × July SNR) pays at MSC#11 (#171)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
+++ b/settlements/skybase/2026-01/skybase_settlement_january_2026.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -511,130 +511,140 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" s="4" t="n">
-        <v>222064.54</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>+ governance_accessibility_rewards (0.01 × SNR 2026-01 = 9218713.81273186308887946403 (sky_total generated sky_total))</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>92187.13812731863</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" s="4" t="n">
+        <v>314251.6781273186</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Sky side</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CoF on utilized (BR × Net_Subs)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>CoF on utilized (BR × Net_Subs)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>+ SDE revenue (Sky-Direct, full to Sky)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="B12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Comparison (Grove-style "Profit to Grove")</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>prime_agent_revenue</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>prime_agent_revenue</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>− CoF (deducted per-venue in display)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-01-01 → 2026-01-31 (31 days)</t>
-        </is>
+      <c r="B17" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pin blocks</t>
+          <t>Period</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ethereum=24358292</t>
+          <t>2026-01-01 → 2026-01-31 (31 days)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Generated</t>
+          <t>Pin blocks</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-05T23:50:42+00:00</t>
+          <t>ethereum=24358292</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Generated</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-08-06T00:02:30+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Pipeline</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>0.1.0</t>
         </is>

</xml_diff>